<commit_message>
Excel files for 2023 ADWR LTSC data
</commit_message>
<xml_diff>
--- a/excel/qry_most_recent_certified_LTSA_credits.xlsx
+++ b/excel/qry_most_recent_certified_LTSA_credits.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="469">
   <si>
     <t xml:space="preserve">AMA</t>
   </si>
@@ -232,12 +232,18 @@
     <t xml:space="preserve">US BUREAU OF RECLAMATION LTSA (TUC AMA)</t>
   </si>
   <si>
+    <t xml:space="preserve">AWBA-MCWA</t>
+  </si>
+  <si>
     <t xml:space="preserve">70-441135.0000</t>
   </si>
   <si>
     <t xml:space="preserve">CITY OF AVONDALE LONG TERM STORAGE ACCOUNT</t>
   </si>
   <si>
+    <t xml:space="preserve">AWBA-INDIAN</t>
+  </si>
+  <si>
     <t xml:space="preserve">70-441247.0000</t>
   </si>
   <si>
@@ -262,25 +268,28 @@
     <t xml:space="preserve">GILA RIVER INDIAN COMMUNITY (PHX) LONG TERM STORAGE ACCOUNT</t>
   </si>
   <si>
+    <t xml:space="preserve">AWBA Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">70-411150.0001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWBA-SNWA (TUCSON AMA) LTSA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">75-411120.0000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAGRD-CDA (TUCSON AMA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">70-441144.0000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CITY OF GOODYEAR LTSA</t>
+  </si>
+  <si>
     <t xml:space="preserve">GRIC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">70-411150.0001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AWBA-SNWA (TUCSON AMA) LTSA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">75-411120.0000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAGRD-CDA (TUCSON AMA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">70-441144.0000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CITY OF GOODYEAR LTSA</t>
   </si>
   <si>
     <t xml:space="preserve">70-441150.0002</t>
@@ -1470,12 +1479,19 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -1504,7 +1520,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1530,6 +1546,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2105,8 +2129,8 @@
       <c r="F28" s="4" t="n">
         <v>178471.78</v>
       </c>
-      <c r="G28" s="3" t="n">
-        <v>2024</v>
+      <c r="G28" s="3" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2165,6 +2189,13 @@
       <c r="G31" s="3" t="n">
         <v>2023</v>
       </c>
+      <c r="H31" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I31" s="6" t="n">
+        <f aca="false">F189+F20</f>
+        <v>256174</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3"/>
@@ -2172,17 +2203,24 @@
         <v>6</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F32" s="4" t="n">
         <v>138260.97</v>
       </c>
       <c r="G32" s="3" t="n">
         <v>2024</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <f aca="false">F39+F60+F69</f>
+        <v>139492.01</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2191,11 +2229,11 @@
         <v>6</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D33" s="3"/>
       <c r="E33" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F33" s="4" t="n">
         <v>137716.46</v>
@@ -2204,7 +2242,7 @@
         <v>2024</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I33" s="6" t="n">
         <f aca="false">F2+F3+F4</f>
@@ -2217,11 +2255,11 @@
         <v>12</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D34" s="3"/>
       <c r="E34" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F34" s="4" t="n">
         <v>130493.52</v>
@@ -2229,10 +2267,10 @@
       <c r="G34" s="3" t="n">
         <v>2023</v>
       </c>
-      <c r="H34" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="I34" s="6" t="n">
+      <c r="H34" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="I34" s="8" t="n">
         <f aca="false">F45+F36+F11</f>
         <v>613846.18</v>
       </c>
@@ -2243,11 +2281,11 @@
         <v>6</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F35" s="4" t="n">
         <v>130253.73</v>
@@ -2256,11 +2294,11 @@
         <v>2024</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I35" s="6" t="n">
-        <f aca="false">F21+F35</f>
-        <v>374659.98</v>
+        <f aca="false">SUM(I31:I34)</f>
+        <v>4416597.27</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2269,11 +2307,11 @@
         <v>12</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F36" s="4" t="n">
         <v>113583.99</v>
@@ -2288,11 +2326,11 @@
         <v>12</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F37" s="4" t="n">
         <v>106065.72</v>
@@ -2307,17 +2345,24 @@
         <v>6</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F38" s="4" t="n">
         <v>95130.62</v>
       </c>
       <c r="G38" s="3" t="n">
         <v>2023</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="I38" s="6" t="n">
+        <f aca="false">F24+F38</f>
+        <v>330601.93</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2326,11 +2371,11 @@
         <v>6</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F39" s="4" t="n">
         <v>88312.95</v>
@@ -2345,11 +2390,11 @@
         <v>6</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F40" s="4" t="n">
         <v>79076.1</v>
@@ -2364,11 +2409,11 @@
         <v>6</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F41" s="4" t="n">
         <v>73782.1</v>
@@ -2383,11 +2428,11 @@
         <v>9</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F42" s="4" t="n">
         <v>72813</v>
@@ -2402,11 +2447,11 @@
         <v>9</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D43" s="3"/>
       <c r="E43" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F43" s="4" t="n">
         <v>71229.85</v>
@@ -2421,11 +2466,11 @@
         <v>6</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="F44" s="4" t="n">
         <v>63225</v>
@@ -2440,11 +2485,11 @@
         <v>6</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D45" s="3"/>
       <c r="E45" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="F45" s="4" t="n">
         <v>60021.16</v>
@@ -2459,11 +2504,11 @@
         <v>9</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D46" s="3"/>
       <c r="E46" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F46" s="4" t="n">
         <v>56682.74</v>
@@ -2478,11 +2523,11 @@
         <v>59</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D47" s="3"/>
       <c r="E47" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="F47" s="4" t="n">
         <v>55000</v>
@@ -2497,11 +2542,11 @@
         <v>12</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D48" s="3"/>
       <c r="E48" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F48" s="4" t="n">
         <v>53210.03</v>
@@ -2516,11 +2561,11 @@
         <v>6</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D49" s="3"/>
       <c r="E49" s="3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F49" s="4" t="n">
         <v>50551.53</v>
@@ -2535,11 +2580,11 @@
         <v>6</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D50" s="3"/>
       <c r="E50" s="3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="F50" s="4" t="n">
         <v>49524.9</v>
@@ -2554,11 +2599,11 @@
         <v>12</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D51" s="3"/>
       <c r="E51" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F51" s="4" t="n">
         <v>44448.61</v>
@@ -2573,11 +2618,11 @@
         <v>12</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D52" s="3"/>
       <c r="E52" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="F52" s="4" t="n">
         <v>43911.87</v>
@@ -2589,14 +2634,14 @@
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3"/>
       <c r="B53" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D53" s="3"/>
       <c r="E53" s="3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F53" s="4" t="n">
         <v>42226.89</v>
@@ -2611,11 +2656,11 @@
         <v>12</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D54" s="3"/>
       <c r="E54" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F54" s="4" t="n">
         <v>38979.66</v>
@@ -2630,11 +2675,11 @@
         <v>12</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D55" s="3"/>
       <c r="E55" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F55" s="4" t="n">
         <v>37735.78</v>
@@ -2649,11 +2694,11 @@
         <v>6</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D56" s="3"/>
       <c r="E56" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F56" s="4" t="n">
         <v>34960.64</v>
@@ -2668,11 +2713,11 @@
         <v>9</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D57" s="3"/>
       <c r="E57" s="3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F57" s="4" t="n">
         <v>34937.92</v>
@@ -2687,11 +2732,11 @@
         <v>9</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D58" s="3"/>
       <c r="E58" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="F58" s="4" t="n">
         <v>34726.42</v>
@@ -2706,11 +2751,11 @@
         <v>12</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D59" s="3"/>
       <c r="E59" s="3" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="F59" s="4" t="n">
         <v>34540.03</v>
@@ -2725,11 +2770,11 @@
         <v>12</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D60" s="3"/>
       <c r="E60" s="3" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F60" s="4" t="n">
         <v>34101.86</v>
@@ -2741,14 +2786,14 @@
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3"/>
       <c r="B61" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D61" s="3"/>
       <c r="E61" s="3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F61" s="4" t="n">
         <v>29298.32</v>
@@ -2760,14 +2805,14 @@
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3"/>
       <c r="B62" s="3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D62" s="3"/>
       <c r="E62" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="F62" s="4" t="n">
         <v>27383</v>
@@ -2782,11 +2827,11 @@
         <v>12</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D63" s="3"/>
       <c r="E63" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="F63" s="4" t="n">
         <v>26817.44</v>
@@ -2801,11 +2846,11 @@
         <v>6</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D64" s="3"/>
       <c r="E64" s="3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="F64" s="4" t="n">
         <v>25933.8</v>
@@ -2820,11 +2865,11 @@
         <v>9</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D65" s="3"/>
       <c r="E65" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="F65" s="4" t="n">
         <v>25500</v>
@@ -2839,11 +2884,11 @@
         <v>12</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D66" s="3"/>
       <c r="E66" s="3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="F66" s="4" t="n">
         <v>25430.74</v>
@@ -2858,11 +2903,11 @@
         <v>12</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D67" s="3"/>
       <c r="E67" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="F67" s="4" t="n">
         <v>19776.95</v>
@@ -2877,11 +2922,11 @@
         <v>6</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D68" s="3"/>
       <c r="E68" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F68" s="4" t="n">
         <v>18071.23</v>
@@ -2896,11 +2941,11 @@
         <v>9</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D69" s="3"/>
       <c r="E69" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F69" s="4" t="n">
         <v>17077.2</v>
@@ -2915,11 +2960,11 @@
         <v>9</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D70" s="3"/>
       <c r="E70" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F70" s="4" t="n">
         <v>16780.14</v>
@@ -2934,11 +2979,11 @@
         <v>6</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D71" s="3"/>
       <c r="E71" s="3" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="F71" s="4" t="n">
         <v>16519.76</v>
@@ -2953,11 +2998,11 @@
         <v>6</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D72" s="3"/>
       <c r="E72" s="3" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F72" s="4" t="n">
         <v>15701.26</v>
@@ -2972,11 +3017,11 @@
         <v>12</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D73" s="3"/>
       <c r="E73" s="3" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="F73" s="4" t="n">
         <v>14955.59</v>
@@ -2991,11 +3036,11 @@
         <v>6</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D74" s="3"/>
       <c r="E74" s="3" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="F74" s="4" t="n">
         <v>14898.57</v>
@@ -3010,11 +3055,11 @@
         <v>6</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D75" s="3"/>
       <c r="E75" s="3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="F75" s="4" t="n">
         <v>14587.85</v>
@@ -3029,11 +3074,11 @@
         <v>9</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D76" s="3"/>
       <c r="E76" s="3" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F76" s="4" t="n">
         <v>12955.49</v>
@@ -3048,11 +3093,11 @@
         <v>12</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D77" s="3"/>
       <c r="E77" s="3" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="F77" s="4" t="n">
         <v>12091.97</v>
@@ -3067,11 +3112,11 @@
         <v>6</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D78" s="3"/>
       <c r="E78" s="3" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="F78" s="4" t="n">
         <v>11850.4</v>
@@ -3086,11 +3131,11 @@
         <v>6</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D79" s="3"/>
       <c r="E79" s="3" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="F79" s="4" t="n">
         <v>11461.62</v>
@@ -3105,11 +3150,11 @@
         <v>6</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D80" s="3"/>
       <c r="E80" s="3" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="F80" s="4" t="n">
         <v>9824.12</v>
@@ -3124,11 +3169,11 @@
         <v>6</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D81" s="3"/>
       <c r="E81" s="3" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="F81" s="4" t="n">
         <v>9500</v>
@@ -3143,11 +3188,11 @@
         <v>9</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D82" s="3"/>
       <c r="E82" s="3" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F82" s="4" t="n">
         <v>8763.9</v>
@@ -3162,11 +3207,11 @@
         <v>12</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D83" s="3"/>
       <c r="E83" s="3" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="F83" s="4" t="n">
         <v>8334.15</v>
@@ -3181,11 +3226,11 @@
         <v>12</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D84" s="3"/>
       <c r="E84" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="F84" s="4" t="n">
         <v>8075.48</v>
@@ -3200,11 +3245,11 @@
         <v>9</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D85" s="3"/>
       <c r="E85" s="3" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F85" s="4" t="n">
         <v>7992.66</v>
@@ -3219,11 +3264,11 @@
         <v>6</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D86" s="3"/>
       <c r="E86" s="3" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="F86" s="4" t="n">
         <v>7618.35</v>
@@ -3238,11 +3283,11 @@
         <v>9</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D87" s="3"/>
       <c r="E87" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F87" s="4" t="n">
         <v>7223.08</v>
@@ -3257,11 +3302,11 @@
         <v>6</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D88" s="3"/>
       <c r="E88" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="F88" s="4" t="n">
         <v>7041.24</v>
@@ -3276,11 +3321,11 @@
         <v>9</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D89" s="3"/>
       <c r="E89" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F89" s="4" t="n">
         <v>7008.26</v>
@@ -3295,11 +3340,11 @@
         <v>59</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D90" s="3"/>
       <c r="E90" s="3" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F90" s="4" t="n">
         <v>7000</v>
@@ -3314,11 +3359,11 @@
         <v>6</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D91" s="3"/>
       <c r="E91" s="3" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="F91" s="4" t="n">
         <v>6969.79</v>
@@ -3333,11 +3378,11 @@
         <v>6</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D92" s="3"/>
       <c r="E92" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F92" s="4" t="n">
         <v>6779.01</v>
@@ -3352,11 +3397,11 @@
         <v>6</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D93" s="3"/>
       <c r="E93" s="3" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F93" s="4" t="n">
         <v>6759</v>
@@ -3371,11 +3416,11 @@
         <v>6</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D94" s="3"/>
       <c r="E94" s="3" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F94" s="4" t="n">
         <v>6532.98</v>
@@ -3390,11 +3435,11 @@
         <v>6</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D95" s="3"/>
       <c r="E95" s="3" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="F95" s="4" t="n">
         <v>6305.99</v>
@@ -3409,11 +3454,11 @@
         <v>6</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D96" s="3"/>
       <c r="E96" s="3" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="F96" s="4" t="n">
         <v>6305</v>
@@ -3428,11 +3473,11 @@
         <v>9</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D97" s="3"/>
       <c r="E97" s="3" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F97" s="4" t="n">
         <v>6192.35</v>
@@ -3447,11 +3492,11 @@
         <v>6</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D98" s="3"/>
       <c r="E98" s="3" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="F98" s="4" t="n">
         <v>5811.01</v>
@@ -3466,11 +3511,11 @@
         <v>6</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D99" s="3"/>
       <c r="E99" s="3" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="F99" s="4" t="n">
         <v>5722.66</v>
@@ -3482,14 +3527,14 @@
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="3"/>
       <c r="B100" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D100" s="3"/>
       <c r="E100" s="3" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F100" s="4" t="n">
         <v>4048.21</v>
@@ -3504,11 +3549,11 @@
         <v>6</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D101" s="3"/>
       <c r="E101" s="3" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="F101" s="4" t="n">
         <v>3933</v>
@@ -3523,11 +3568,11 @@
         <v>12</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D102" s="3"/>
       <c r="E102" s="3" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="F102" s="4" t="n">
         <v>3923.15</v>
@@ -3542,11 +3587,11 @@
         <v>6</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="D103" s="3"/>
       <c r="E103" s="3" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F103" s="4" t="n">
         <v>3800.57</v>
@@ -3561,11 +3606,11 @@
         <v>9</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D104" s="3"/>
       <c r="E104" s="3" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F104" s="4" t="n">
         <v>3749.08</v>
@@ -3580,11 +3625,11 @@
         <v>12</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D105" s="3"/>
       <c r="E105" s="3" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F105" s="4" t="n">
         <v>3735.29</v>
@@ -3599,11 +3644,11 @@
         <v>6</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D106" s="3"/>
       <c r="E106" s="3" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="F106" s="4" t="n">
         <v>3575.24</v>
@@ -3618,11 +3663,11 @@
         <v>6</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="D107" s="3"/>
       <c r="E107" s="3" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F107" s="4" t="n">
         <v>3421.41</v>
@@ -3637,11 +3682,11 @@
         <v>9</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D108" s="3"/>
       <c r="E108" s="3" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="F108" s="4" t="n">
         <v>3028.42</v>
@@ -3656,11 +3701,11 @@
         <v>12</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D109" s="3"/>
       <c r="E109" s="3" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="F109" s="4" t="n">
         <v>2797.8</v>
@@ -3675,11 +3720,11 @@
         <v>9</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D110" s="3"/>
       <c r="E110" s="3" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="F110" s="4" t="n">
         <v>2752.22</v>
@@ -3694,11 +3739,11 @@
         <v>6</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D111" s="3"/>
       <c r="E111" s="3" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="F111" s="4" t="n">
         <v>2310.34</v>
@@ -3713,11 +3758,11 @@
         <v>12</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D112" s="3"/>
       <c r="E112" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="F112" s="4" t="n">
         <v>2033.4</v>
@@ -3732,11 +3777,11 @@
         <v>6</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D113" s="3"/>
       <c r="E113" s="3" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="F113" s="4" t="n">
         <v>2000</v>
@@ -3748,14 +3793,14 @@
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="3"/>
       <c r="B114" s="3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="D114" s="3"/>
       <c r="E114" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="F114" s="4" t="n">
         <v>1933.29</v>
@@ -3767,16 +3812,16 @@
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="3"/>
       <c r="B115" s="3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="F115" s="4" t="n">
         <v>1903.92</v>
@@ -3791,11 +3836,11 @@
         <v>6</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="D116" s="3"/>
       <c r="E116" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="F116" s="4" t="n">
         <v>1902.48</v>
@@ -3810,11 +3855,11 @@
         <v>9</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D117" s="3"/>
       <c r="E117" s="3" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="F117" s="4" t="n">
         <v>1886.89</v>
@@ -3829,11 +3874,11 @@
         <v>12</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="D118" s="3"/>
       <c r="E118" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="F118" s="4" t="n">
         <v>1833.8</v>
@@ -3848,11 +3893,11 @@
         <v>9</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="D119" s="3"/>
       <c r="E119" s="3" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="F119" s="4" t="n">
         <v>1795.56</v>
@@ -3867,11 +3912,11 @@
         <v>12</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D120" s="3"/>
       <c r="E120" s="3" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="F120" s="4" t="n">
         <v>1750</v>
@@ -3883,14 +3928,14 @@
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="3"/>
       <c r="B121" s="3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="D121" s="3"/>
       <c r="E121" s="3" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="F121" s="4" t="n">
         <v>1713.7</v>
@@ -3905,11 +3950,11 @@
         <v>6</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="D122" s="3"/>
       <c r="E122" s="3" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="F122" s="4" t="n">
         <v>1566.32</v>
@@ -3924,11 +3969,11 @@
         <v>6</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="D123" s="3"/>
       <c r="E123" s="3" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="F123" s="4" t="n">
         <v>1488.07</v>
@@ -3943,11 +3988,11 @@
         <v>9</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D124" s="3"/>
       <c r="E124" s="3" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="F124" s="4" t="n">
         <v>1464.16</v>
@@ -3962,11 +4007,11 @@
         <v>12</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D125" s="3"/>
       <c r="E125" s="3" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F125" s="4" t="n">
         <v>1429</v>
@@ -3981,11 +4026,11 @@
         <v>9</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="D126" s="3"/>
       <c r="E126" s="3" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="F126" s="4" t="n">
         <v>1387</v>
@@ -3997,14 +4042,14 @@
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="3"/>
       <c r="B127" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="D127" s="3"/>
       <c r="E127" s="3" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="F127" s="4" t="n">
         <v>1330</v>
@@ -4019,11 +4064,11 @@
         <v>6</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="D128" s="3"/>
       <c r="E128" s="3" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="F128" s="4" t="n">
         <v>1320</v>
@@ -4035,14 +4080,14 @@
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="3"/>
       <c r="B129" s="3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="D129" s="3"/>
       <c r="E129" s="3" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F129" s="4" t="n">
         <v>1220.14</v>
@@ -4057,11 +4102,11 @@
         <v>6</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="D130" s="3"/>
       <c r="E130" s="3" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="F130" s="4" t="n">
         <v>1080</v>
@@ -4076,11 +4121,11 @@
         <v>6</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="D131" s="3"/>
       <c r="E131" s="3" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="F131" s="4" t="n">
         <v>1072</v>
@@ -4095,11 +4140,11 @@
         <v>6</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="D132" s="3"/>
       <c r="E132" s="3" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="F132" s="4" t="n">
         <v>950</v>
@@ -4114,11 +4159,11 @@
         <v>6</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D133" s="3"/>
       <c r="E133" s="3" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="F133" s="4" t="n">
         <v>796.98</v>
@@ -4133,11 +4178,11 @@
         <v>6</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="D134" s="3"/>
       <c r="E134" s="3" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="F134" s="4" t="n">
         <v>658.56</v>
@@ -4152,11 +4197,11 @@
         <v>6</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="D135" s="3"/>
       <c r="E135" s="3" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="F135" s="4" t="n">
         <v>621</v>
@@ -4171,11 +4216,11 @@
         <v>6</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="D136" s="3"/>
       <c r="E136" s="3" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="F136" s="4" t="n">
         <v>620.56</v>
@@ -4190,11 +4235,11 @@
         <v>6</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="D137" s="3"/>
       <c r="E137" s="3" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F137" s="4" t="n">
         <v>535.55</v>
@@ -4206,14 +4251,14 @@
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="3"/>
       <c r="B138" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D138" s="3"/>
       <c r="E138" s="3" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="F138" s="4" t="n">
         <v>527.62</v>
@@ -4228,11 +4273,11 @@
         <v>12</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="D139" s="3"/>
       <c r="E139" s="3" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="F139" s="4" t="n">
         <v>518</v>
@@ -4244,16 +4289,16 @@
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="3"/>
       <c r="B140" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="F140" s="4" t="n">
         <v>503.5</v>
@@ -4268,11 +4313,11 @@
         <v>6</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="D141" s="3"/>
       <c r="E141" s="3" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F141" s="4" t="n">
         <v>481.24</v>
@@ -4287,11 +4332,11 @@
         <v>6</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D142" s="3"/>
       <c r="E142" s="3" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F142" s="4" t="n">
         <v>443</v>
@@ -4306,11 +4351,11 @@
         <v>9</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="D143" s="3"/>
       <c r="E143" s="3" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="F143" s="4" t="n">
         <v>347</v>
@@ -4325,11 +4370,11 @@
         <v>6</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D144" s="3"/>
       <c r="E144" s="3" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F144" s="4" t="n">
         <v>334.4</v>
@@ -4344,11 +4389,11 @@
         <v>6</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="D145" s="3"/>
       <c r="E145" s="3" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="F145" s="4" t="n">
         <v>308.83</v>
@@ -4363,11 +4408,11 @@
         <v>6</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="D146" s="3"/>
       <c r="E146" s="3" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="F146" s="4" t="n">
         <v>218</v>
@@ -4382,11 +4427,11 @@
         <v>9</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="D147" s="3"/>
       <c r="E147" s="3" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="F147" s="4" t="n">
         <v>214.77</v>
@@ -4401,11 +4446,11 @@
         <v>6</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="D148" s="3"/>
       <c r="E148" s="3" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="F148" s="4" t="n">
         <v>168</v>
@@ -4420,11 +4465,11 @@
         <v>6</v>
       </c>
       <c r="C149" s="3" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="D149" s="3"/>
       <c r="E149" s="3" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="F149" s="4" t="n">
         <v>165.63</v>
@@ -4439,11 +4484,11 @@
         <v>6</v>
       </c>
       <c r="C150" s="3" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="D150" s="3"/>
       <c r="E150" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="F150" s="4" t="n">
         <v>162.5</v>
@@ -4458,11 +4503,11 @@
         <v>9</v>
       </c>
       <c r="C151" s="3" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="D151" s="3"/>
       <c r="E151" s="3" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="F151" s="4" t="n">
         <v>130.49</v>
@@ -4477,11 +4522,11 @@
         <v>6</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D152" s="3"/>
       <c r="E152" s="3" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="F152" s="4" t="n">
         <v>111.21</v>
@@ -4496,11 +4541,11 @@
         <v>12</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="D153" s="3"/>
       <c r="E153" s="3" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="F153" s="4" t="n">
         <v>90.09</v>
@@ -4515,11 +4560,11 @@
         <v>9</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="D154" s="3"/>
       <c r="E154" s="3" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="F154" s="4" t="n">
         <v>89.99</v>
@@ -4534,11 +4579,11 @@
         <v>9</v>
       </c>
       <c r="C155" s="3" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="D155" s="3"/>
       <c r="E155" s="3" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="F155" s="4" t="n">
         <v>84.29</v>
@@ -4550,14 +4595,14 @@
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="3"/>
       <c r="B156" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C156" s="3" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="D156" s="3"/>
       <c r="E156" s="3" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="F156" s="4" t="n">
         <v>56.33</v>
@@ -4572,11 +4617,11 @@
         <v>6</v>
       </c>
       <c r="C157" s="3" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="D157" s="3"/>
       <c r="E157" s="3" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="F157" s="4" t="n">
         <v>50.1</v>
@@ -4591,11 +4636,11 @@
         <v>6</v>
       </c>
       <c r="C158" s="3" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="D158" s="3"/>
       <c r="E158" s="3" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F158" s="4" t="n">
         <v>50</v>
@@ -4610,11 +4655,11 @@
         <v>12</v>
       </c>
       <c r="C159" s="3" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="D159" s="3"/>
       <c r="E159" s="3" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F159" s="4" t="n">
         <v>50</v>
@@ -4629,11 +4674,11 @@
         <v>6</v>
       </c>
       <c r="C160" s="3" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="D160" s="3"/>
       <c r="E160" s="3" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="F160" s="4" t="n">
         <v>49.72</v>
@@ -4648,11 +4693,11 @@
         <v>6</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="D161" s="3"/>
       <c r="E161" s="3" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="F161" s="4" t="n">
         <v>49.59</v>
@@ -4667,11 +4712,11 @@
         <v>6</v>
       </c>
       <c r="C162" s="3" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D162" s="3"/>
       <c r="E162" s="3" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F162" s="4" t="n">
         <v>47.29</v>
@@ -4686,11 +4731,11 @@
         <v>6</v>
       </c>
       <c r="C163" s="3" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="D163" s="3"/>
       <c r="E163" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="F163" s="4" t="n">
         <v>45.23</v>
@@ -4705,11 +4750,11 @@
         <v>6</v>
       </c>
       <c r="C164" s="3" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="D164" s="3"/>
       <c r="E164" s="3" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="F164" s="4" t="n">
         <v>42.35</v>
@@ -4724,11 +4769,11 @@
         <v>6</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="D165" s="3"/>
       <c r="E165" s="3" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="F165" s="4" t="n">
         <v>39.88</v>
@@ -4743,11 +4788,11 @@
         <v>6</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="D166" s="3"/>
       <c r="E166" s="3" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="F166" s="4" t="n">
         <v>35.12</v>
@@ -4762,11 +4807,11 @@
         <v>6</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="D167" s="3"/>
       <c r="E167" s="3" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="F167" s="4" t="n">
         <v>33.56</v>
@@ -4781,11 +4826,11 @@
         <v>6</v>
       </c>
       <c r="C168" s="3" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="D168" s="3"/>
       <c r="E168" s="3" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="F168" s="4" t="n">
         <v>33.46</v>
@@ -4800,11 +4845,11 @@
         <v>9</v>
       </c>
       <c r="C169" s="3" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="D169" s="3"/>
       <c r="E169" s="3" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="F169" s="4" t="n">
         <v>30.24</v>
@@ -4819,11 +4864,11 @@
         <v>6</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="D170" s="3"/>
       <c r="E170" s="3" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="F170" s="4" t="n">
         <v>28.98</v>
@@ -4838,11 +4883,11 @@
         <v>6</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="D171" s="3"/>
       <c r="E171" s="3" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="F171" s="4" t="n">
         <v>26</v>
@@ -4857,11 +4902,11 @@
         <v>6</v>
       </c>
       <c r="C172" s="3" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D172" s="3"/>
       <c r="E172" s="3" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="F172" s="4" t="n">
         <v>23.28</v>
@@ -4876,11 +4921,11 @@
         <v>6</v>
       </c>
       <c r="C173" s="3" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="D173" s="3"/>
       <c r="E173" s="3" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="F173" s="4" t="n">
         <v>20</v>
@@ -4895,11 +4940,11 @@
         <v>6</v>
       </c>
       <c r="C174" s="3" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="D174" s="3"/>
       <c r="E174" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="F174" s="4" t="n">
         <v>12</v>
@@ -4914,11 +4959,11 @@
         <v>6</v>
       </c>
       <c r="C175" s="3" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="D175" s="3"/>
       <c r="E175" s="3" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="F175" s="4" t="n">
         <v>10.5</v>
@@ -4933,11 +4978,11 @@
         <v>12</v>
       </c>
       <c r="C176" s="3" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="D176" s="3"/>
       <c r="E176" s="3" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="F176" s="4" t="n">
         <v>7.56</v>
@@ -4952,11 +4997,11 @@
         <v>6</v>
       </c>
       <c r="C177" s="3" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="D177" s="3"/>
       <c r="E177" s="3" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="F177" s="4" t="n">
         <v>5.64</v>
@@ -4971,11 +5016,11 @@
         <v>12</v>
       </c>
       <c r="C178" s="3" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="D178" s="3"/>
       <c r="E178" s="3" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="F178" s="4" t="n">
         <v>5.39</v>
@@ -4990,11 +5035,11 @@
         <v>6</v>
       </c>
       <c r="C179" s="3" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="D179" s="3"/>
       <c r="E179" s="3" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="F179" s="4" t="n">
         <v>5</v>
@@ -5009,11 +5054,11 @@
         <v>6</v>
       </c>
       <c r="C180" s="3" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="D180" s="3"/>
       <c r="E180" s="3" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="F180" s="4" t="n">
         <v>3</v>
@@ -5028,11 +5073,11 @@
         <v>6</v>
       </c>
       <c r="C181" s="3" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="D181" s="3"/>
       <c r="E181" s="3" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="F181" s="4" t="n">
         <v>2.75</v>
@@ -5047,11 +5092,11 @@
         <v>6</v>
       </c>
       <c r="C182" s="3" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="D182" s="3"/>
       <c r="E182" s="3" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="F182" s="4" t="n">
         <v>1</v>
@@ -5066,11 +5111,11 @@
         <v>6</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="D183" s="3"/>
       <c r="E183" s="3" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="F183" s="4" t="n">
         <v>1</v>
@@ -5085,11 +5130,11 @@
         <v>6</v>
       </c>
       <c r="C184" s="3" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="D184" s="3"/>
       <c r="E184" s="3" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="F184" s="4" t="n">
         <v>1</v>
@@ -5104,11 +5149,11 @@
         <v>12</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="D185" s="3"/>
       <c r="E185" s="3" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="F185" s="4" t="n">
         <v>0.75</v>
@@ -5123,11 +5168,11 @@
         <v>12</v>
       </c>
       <c r="C186" s="3" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="D186" s="3"/>
       <c r="E186" s="3" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="F186" s="4" t="n">
         <v>0.04</v>
@@ -5139,14 +5184,14 @@
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="3"/>
       <c r="B187" s="3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C187" s="3" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="D187" s="3"/>
       <c r="E187" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F187" s="4" t="n">
         <v>0</v>
@@ -5161,11 +5206,11 @@
         <v>6</v>
       </c>
       <c r="C188" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="D188" s="3"/>
       <c r="E188" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="F188" s="4" t="n">
         <v>0</v>
@@ -5180,11 +5225,11 @@
         <v>6</v>
       </c>
       <c r="C189" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="D189" s="3"/>
       <c r="E189" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="F189" s="4" t="n">
         <v>0</v>
@@ -5199,11 +5244,11 @@
         <v>6</v>
       </c>
       <c r="C190" s="3" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="D190" s="3"/>
       <c r="E190" s="3" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="F190" s="4" t="n">
         <v>0</v>
@@ -5218,11 +5263,11 @@
         <v>6</v>
       </c>
       <c r="C191" s="3" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="D191" s="3"/>
       <c r="E191" s="3" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="F191" s="4" t="n">
         <v>0</v>
@@ -5237,11 +5282,11 @@
         <v>6</v>
       </c>
       <c r="C192" s="3" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="D192" s="3"/>
       <c r="E192" s="3" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="F192" s="4" t="n">
         <v>0</v>
@@ -5256,11 +5301,11 @@
         <v>6</v>
       </c>
       <c r="C193" s="3" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="D193" s="3"/>
       <c r="E193" s="3" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="F193" s="4" t="n">
         <v>0</v>
@@ -5275,11 +5320,11 @@
         <v>6</v>
       </c>
       <c r="C194" s="3" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="D194" s="3"/>
       <c r="E194" s="3" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="F194" s="4" t="n">
         <v>0</v>
@@ -5294,11 +5339,11 @@
         <v>6</v>
       </c>
       <c r="C195" s="3" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="D195" s="3"/>
       <c r="E195" s="3" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="F195" s="4" t="n">
         <v>0</v>
@@ -5313,11 +5358,11 @@
         <v>6</v>
       </c>
       <c r="C196" s="3" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="D196" s="3"/>
       <c r="E196" s="3" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="F196" s="4" t="n">
         <v>0</v>
@@ -5332,11 +5377,11 @@
         <v>6</v>
       </c>
       <c r="C197" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="D197" s="3"/>
       <c r="E197" s="3" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="F197" s="4" t="n">
         <v>0</v>
@@ -5351,11 +5396,11 @@
         <v>6</v>
       </c>
       <c r="C198" s="3" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="D198" s="3"/>
       <c r="E198" s="3" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="F198" s="4" t="n">
         <v>0</v>
@@ -5370,11 +5415,11 @@
         <v>6</v>
       </c>
       <c r="C199" s="3" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="D199" s="3"/>
       <c r="E199" s="3" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="F199" s="4" t="n">
         <v>0</v>
@@ -5389,11 +5434,11 @@
         <v>6</v>
       </c>
       <c r="C200" s="3" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="D200" s="3"/>
       <c r="E200" s="3" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="F200" s="4" t="n">
         <v>0</v>
@@ -5408,11 +5453,11 @@
         <v>6</v>
       </c>
       <c r="C201" s="3" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="D201" s="3"/>
       <c r="E201" s="3" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="F201" s="4" t="n">
         <v>0</v>
@@ -5427,11 +5472,11 @@
         <v>6</v>
       </c>
       <c r="C202" s="3" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="D202" s="3"/>
       <c r="E202" s="3" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="F202" s="4" t="n">
         <v>0</v>
@@ -5446,11 +5491,11 @@
         <v>6</v>
       </c>
       <c r="C203" s="3" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="D203" s="3"/>
       <c r="E203" s="3" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="F203" s="4" t="n">
         <v>0</v>
@@ -5465,11 +5510,11 @@
         <v>6</v>
       </c>
       <c r="C204" s="3" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="D204" s="3"/>
       <c r="E204" s="3" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="F204" s="4" t="n">
         <v>0</v>
@@ -5484,11 +5529,11 @@
         <v>6</v>
       </c>
       <c r="C205" s="3" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="D205" s="3"/>
       <c r="E205" s="3" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="F205" s="4" t="n">
         <v>0</v>
@@ -5503,11 +5548,11 @@
         <v>9</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="D206" s="3"/>
       <c r="E206" s="3" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="F206" s="4" t="n">
         <v>0</v>
@@ -5522,11 +5567,11 @@
         <v>9</v>
       </c>
       <c r="C207" s="3" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="D207" s="3"/>
       <c r="E207" s="3" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="F207" s="4" t="n">
         <v>0</v>
@@ -5541,11 +5586,11 @@
         <v>9</v>
       </c>
       <c r="C208" s="3" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="D208" s="3"/>
       <c r="E208" s="3" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="F208" s="4" t="n">
         <v>0</v>
@@ -5560,11 +5605,11 @@
         <v>9</v>
       </c>
       <c r="C209" s="3" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="D209" s="3"/>
       <c r="E209" s="3" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="F209" s="4" t="n">
         <v>0</v>
@@ -5579,11 +5624,11 @@
         <v>9</v>
       </c>
       <c r="C210" s="3" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="D210" s="3"/>
       <c r="E210" s="3" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="F210" s="4" t="n">
         <v>0</v>
@@ -5598,11 +5643,11 @@
         <v>9</v>
       </c>
       <c r="C211" s="3" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="D211" s="3"/>
       <c r="E211" s="3" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="F211" s="4" t="n">
         <v>0</v>
@@ -5617,11 +5662,11 @@
         <v>9</v>
       </c>
       <c r="C212" s="3" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="D212" s="3"/>
       <c r="E212" s="3" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="F212" s="4" t="n">
         <v>0</v>
@@ -5636,11 +5681,11 @@
         <v>9</v>
       </c>
       <c r="C213" s="3" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="D213" s="3"/>
       <c r="E213" s="3" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="F213" s="4" t="n">
         <v>0</v>
@@ -5652,16 +5697,16 @@
     <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="3"/>
       <c r="B214" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C214" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D214" s="3" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="E214" s="3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F214" s="4" t="n">
         <v>0</v>
@@ -5676,11 +5721,11 @@
         <v>12</v>
       </c>
       <c r="C215" s="3" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="D215" s="3"/>
       <c r="E215" s="3" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="F215" s="4" t="n">
         <v>0</v>
@@ -5695,11 +5740,11 @@
         <v>12</v>
       </c>
       <c r="C216" s="3" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D216" s="3"/>
       <c r="E216" s="3" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="F216" s="4" t="n">
         <v>0</v>
@@ -5714,11 +5759,11 @@
         <v>12</v>
       </c>
       <c r="C217" s="3" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="D217" s="3"/>
       <c r="E217" s="3" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="F217" s="4" t="n">
         <v>0</v>
@@ -5733,11 +5778,11 @@
         <v>12</v>
       </c>
       <c r="C218" s="3" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="D218" s="3"/>
       <c r="E218" s="3" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="F218" s="4" t="n">
         <v>0</v>
@@ -5752,11 +5797,11 @@
         <v>12</v>
       </c>
       <c r="C219" s="3" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D219" s="3"/>
       <c r="E219" s="3" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="F219" s="4" t="n">
         <v>0</v>
@@ -5771,11 +5816,11 @@
         <v>12</v>
       </c>
       <c r="C220" s="3" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="D220" s="3"/>
       <c r="E220" s="3" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="F220" s="4" t="n">
         <v>0</v>
@@ -5790,11 +5835,11 @@
         <v>12</v>
       </c>
       <c r="C221" s="3" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="D221" s="3"/>
       <c r="E221" s="3" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="F221" s="4" t="n">
         <v>-8.82</v>
@@ -5805,9 +5850,9 @@
     </row>
     <row r="222" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="3" t="s">
-        <v>453</v>
-      </c>
-      <c r="F222" s="7" t="n">
+        <v>456</v>
+      </c>
+      <c r="F222" s="9" t="n">
         <f aca="false">SUM(F2:F221)</f>
         <v>14853766.95</v>
       </c>
@@ -5827,11 +5872,11 @@
         <v>6</v>
       </c>
       <c r="C224" s="3" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="D224" s="3"/>
       <c r="E224" s="3" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="F224" s="3"/>
       <c r="G224" s="3"/>
@@ -5842,11 +5887,11 @@
         <v>6</v>
       </c>
       <c r="C225" s="3" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="D225" s="3"/>
       <c r="E225" s="3" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="F225" s="3"/>
       <c r="G225" s="3"/>
@@ -5857,11 +5902,11 @@
         <v>6</v>
       </c>
       <c r="C226" s="3" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="D226" s="3"/>
       <c r="E226" s="3" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="F226" s="3"/>
       <c r="G226" s="3"/>
@@ -5872,11 +5917,11 @@
         <v>6</v>
       </c>
       <c r="C227" s="3" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="D227" s="3"/>
       <c r="E227" s="3" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="F227" s="3"/>
       <c r="G227" s="3"/>
@@ -5884,14 +5929,14 @@
     <row r="228" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="3"/>
       <c r="B228" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C228" s="3" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="D228" s="3"/>
       <c r="E228" s="3" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F228" s="3"/>
       <c r="G228" s="3"/>
@@ -5902,11 +5947,11 @@
         <v>12</v>
       </c>
       <c r="C229" s="3" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="D229" s="3"/>
       <c r="E229" s="3" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="F229" s="3"/>
       <c r="G229" s="3"/>

</xml_diff>